<commit_message>
RTM Synchronized and expanded
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/API Testing/Documentation/Automation Exercise API Test Cases.xlsx
+++ b/Automation Exercise Project/API Testing/Documentation/Automation Exercise API Test Cases.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R88eb4802add84d55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Test Cases" sheetId="2" r:id="Rf103d8236b194875"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R8a30730ab5c04d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R4a2e1b2f193b430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Raa6bd72c3b12435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Test Cases" sheetId="2" r:id="R3aa19c111ecd4857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="Re5a15a69522645c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R6aaf1d6907b249b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Summary" sheetId="5" r:id="R22bd8e4fb33f4b95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,9 +17,6 @@
     <x:t xml:space="preserve">Automation Exercise — API Test Execution Overview</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Postman API testing mapped to REQ-API-001 through REQ-API-014 | Portfolio execution workbook</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Total API Cases</x:t>
   </x:si>
   <x:si>
@@ -172,24 +170,6 @@
 5. Verify responseCode and products in the JSON body.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">. Response body contained responseCode 200 and a populated products array with product IDs, names, prices, brands, and categories.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Pass</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KM</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">../Execution Results/Screenshots/API-PRODUCT-001.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NA</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 1.81 KB.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-PRODUCT-002</x:t>
   </x:si>
   <x:si>
@@ -217,15 +197,6 @@
 4. Compare the response with the expected method-not-supported response.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">. Response body contained responseCode 405. "message": "This request method is not supported."</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">km</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-PRODUCT-002.png</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-BRAND-001</x:t>
   </x:si>
   <x:si>
@@ -244,15 +215,6 @@
 4. Verify the status and brands list.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> Response body contained responseCode 200 and a populated products array with all brands.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-BRAND-001.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 1.06 KB.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-BRAND-002</x:t>
   </x:si>
   <x:si>
@@ -271,15 +233,6 @@
 4. Verify the method-not-supported response.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">"responseCode": 405, "message": "This request method is not supported."}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-BRAND-002.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 912 B.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-SEARCH-001</x:t>
   </x:si>
   <x:si>
@@ -304,15 +257,6 @@
 4. Verify status and searched products.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> Response body contained responseCode 200 and a populated products array with all "tops".</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-SEARCH-001.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 1.32 KB.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-SEARCH-002</x:t>
   </x:si>
   <x:si>
@@ -331,12 +275,6 @@
 4. Verify the missing-parameter response.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> Response body contained responseCode 200 and a populated products array with all products</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-SEARCH-002.png</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-AUTH-001</x:t>
   </x:si>
   <x:si>
@@ -364,15 +302,6 @@
 4. Verify status and User exists message.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">{"responseCode": 200, "message": "User exists!"}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-AUTH-001.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 848 B.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-AUTH-002</x:t>
   </x:si>
   <x:si>
@@ -394,15 +323,6 @@
 4. Verify the missing-parameter response.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">{"responseCode": 400, "message": "Bad request, email or password parameter is missing in POST request."}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-AUTH-002.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 927 B</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-AUTH-003</x:t>
   </x:si>
   <x:si>
@@ -421,15 +341,6 @@
 4. Verify the method-not-supported response.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">{"responseCode": 405, "message": "This request method is not supported."}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-AUTH-003.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 908 B</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-AUTH-004</x:t>
   </x:si>
   <x:si>
@@ -451,15 +362,6 @@
 4. Verify status and User not found message.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">{"responseCode": 404, "message": "User not found!"}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-AUTH-004.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 881 B</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-ACCOUNT-001</x:t>
   </x:si>
   <x:si>
@@ -484,15 +386,6 @@
 4. Preserve sanitized evidence.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">{"responseCode": 201, "message": "User created!"}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-ACCOUNT-001.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Use only a disposable QA account.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-ACCOUNT-002</x:t>
   </x:si>
   <x:si>
@@ -516,15 +409,6 @@
 3. Verify status and Account deleted message.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">{"responseCode": 200, "message": "Account deleted!"}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-ACCOUNT-002.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 854 B</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-ACCOUNT-003</x:t>
   </x:si>
   <x:si>
@@ -545,12 +429,6 @@
 3. Verify status and User updated message.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">{"responseCode": 200, "message": "User updated!"}</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-ACCOUNT-003.png</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API-ACCOUNT-004</x:t>
   </x:si>
   <x:si>
@@ -574,15 +452,6 @@
 3. Verify status and returned user details.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">HTTP 200 with User Detail JSON.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">..\Execution Results\Screenshots\API-ACCOUNT-004.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Initial manual Postman execution. Response size displayed as 1.06 B</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">API Test Workbook — Usage Guide</x:t>
   </x:si>
   <x:si>
@@ -707,6 +576,9 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Statuses</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Pass</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Fail</x:t>
@@ -728,7 +600,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -794,8 +666,54 @@
       <x:sz val="10"/>
       <x:name val="Arial Unicode MS"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF16324F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17603A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF16324F"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17603A"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -830,6 +748,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B3558"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1386B8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2C94C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9F2E6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -936,7 +879,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -1092,6 +1035,73 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -1773,8 +1783,8 @@
       <x:c r="N1" s="11"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="12" t="s">
-        <x:v>1</x:v>
+      <x:c r="A2" s="12" t="str">
+        <x:v>Professional API QA repository | 14 official requirements | historical Postman baseline plus current automated verification</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -1792,22 +1802,22 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="13" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="14"/>
       <x:c r="C4" s="15"/>
       <x:c r="E4" s="13" t="s">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F4" s="14"/>
       <x:c r="G4" s="15"/>
       <x:c r="I4" s="13" t="s">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J4" s="14"/>
       <x:c r="K4" s="15"/>
       <x:c r="M4" s="13" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N4" s="15"/>
     </x:row>
@@ -1820,7 +1830,7 @@
       <x:c r="C5" s="18"/>
       <x:c r="E5" s="16" t="n">
         <x:f>COUNTIF('API Test Cases'!S8:S21,"Pass")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F5" s="17"/>
       <x:c r="G5" s="18"/>
@@ -1851,19 +1861,19 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="s">
+      <x:c r="C8" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C8" s="2" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="s">
+      <x:c r="F8" s="22" t="s">
         <x:v>8</x:v>
-      </x:c>
-      <x:c r="F8" s="22" t="s">
-        <x:v>9</x:v>
       </x:c>
       <x:c r="G8" s="22"/>
       <x:c r="H8" s="22"/>
@@ -1876,7 +1886,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="45" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B9" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A9)</x:f>
@@ -1891,7 +1901,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="23" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G9" s="24"/>
       <x:c r="H9" s="24"/>
@@ -1904,7 +1914,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="45" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B10" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A10)</x:f>
@@ -1930,7 +1940,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="45" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B11" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A11)</x:f>
@@ -1938,11 +1948,11 @@
       </x:c>
       <x:c r="C11" s="45" t="n">
         <x:f>COUNTIFS('API Test Cases'!C8:C21,A11,'API Test Cases'!S8:S21,"Pass")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D11" s="45" t="n">
         <x:f>B11-C11</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="26"/>
       <x:c r="G11" s="27"/>
@@ -1956,7 +1966,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B12" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A12)</x:f>
@@ -1982,7 +1992,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B13" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A13)</x:f>
@@ -2056,7 +2066,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="11" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B1" s="11"/>
       <x:c r="C1" s="11"/>
@@ -2112,7 +2122,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="32" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B4" s="33"/>
       <x:c r="C4" s="33"/>
@@ -2122,7 +2132,7 @@
       <x:c r="G4" s="33"/>
       <x:c r="H4" s="34"/>
       <x:c r="J4" s="38" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="K4" s="39"/>
       <x:c r="L4" s="39"/>
@@ -2166,117 +2176,117 @@
     </x:row>
     <x:row r="7" ht="44" customHeight="1">
       <x:c r="A7" s="4" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B7" s="4" t="s">
+      <x:c r="C7" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C7" s="4" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D7" s="4" t="s">
+      <x:c r="E7" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E7" s="4" t="s">
+      <x:c r="F7" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="s">
+      <x:c r="G7" s="4" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="G7" s="4" t="s">
+      <x:c r="H7" s="4" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="H7" s="4" t="s">
+      <x:c r="I7" s="4" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="I7" s="4" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="J7" s="4" t="s">
+      <x:c r="K7" s="4" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="K7" s="4" t="s">
+      <x:c r="L7" s="4" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="L7" s="4" t="s">
+      <x:c r="M7" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="M7" s="4" t="s">
+      <x:c r="N7" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="N7" s="4" t="s">
+      <x:c r="O7" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="O7" s="4" t="s">
+      <x:c r="P7" s="4" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="P7" s="4" t="s">
+      <x:c r="Q7" s="4" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="Q7" s="4" t="s">
+      <x:c r="R7" s="4" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="R7" s="4" t="s">
+      <x:c r="S7" s="4" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="S7" s="4" t="s">
+      <x:c r="T7" s="4" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="T7" s="4" t="s">
+      <x:c r="U7" s="4" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="U7" s="4" t="s">
+      <x:c r="V7" s="4" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="V7" s="4" t="s">
+      <x:c r="W7" s="4" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="W7" s="4" t="s">
+      <x:c r="X7" s="4" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="X7" s="4" t="s">
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="47" t="s">
         <x:v>40</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="78.5" customHeight="1">
-      <x:c r="A8" s="47" t="s">
+      <x:c r="B8" s="50" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B8" s="50" t="s">
+      <x:c r="C8" s="47" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="C8" s="47" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D8" s="47" t="s">
+      <x:c r="E8" s="47" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="E8" s="47" t="s">
+      <x:c r="F8" s="46" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="F8" s="46" t="s">
+      <x:c r="G8" s="47" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="G8" s="47" t="s">
+      <x:c r="H8" s="47" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="H8" s="47" t="s">
+      <x:c r="I8" s="47" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="I8" s="47" t="s">
+      <x:c r="J8" s="47" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="K8" s="46" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="L8" s="46" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="J8" s="47" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="K8" s="46" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="L8" s="46" t="s">
+      <x:c r="M8" s="46" t="s">
         <x:v>49</x:v>
-      </x:c>
-      <x:c r="M8" s="46" t="s">
-        <x:v>50</x:v>
       </x:c>
       <x:c r="N8" s="47">
         <x:v>200</x:v>
@@ -2284,73 +2294,74 @@
       <x:c r="O8" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 200; a non-empty products array containing product details.</x:v>
       </x:c>
-      <x:c r="P8" s="47">
+      <x:c r="P8" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q8" s="46" t="s">
+      <x:c r="Q8" s="46" t="str">
+        <x:v>200 | products list returned</x:v>
+      </x:c>
+      <x:c r="R8" s="47" t="n">
+        <x:v>616</x:v>
+      </x:c>
+      <x:c r="S8" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T8" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U8" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V8" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-PRODUCT-001.png
+..\..\Automation\Execution Evidence\API-PRODUCT-001.png</x:v>
+      </x:c>
+      <x:c r="W8" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X8" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="47" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B9" s="50" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="R8" s="47">
-        <x:v>616</x:v>
-      </x:c>
-      <x:c r="S8" s="47" t="s">
+      <x:c r="C9" s="47" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D9" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="T8" s="47" t="s">
+      <x:c r="E9" s="47" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="U8" s="49">
-        <x:v>46234.666666666664</x:v>
-      </x:c>
-      <x:c r="V8" s="50" t="s">
+      <x:c r="F9" s="46" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="W8" s="47" t="s">
+      <x:c r="G9" s="47" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="X8" s="46" t="s">
+      <x:c r="H9" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="I9" s="47" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="J9" s="47" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="K9" s="46" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="L9" s="46" t="s">
         <x:v>56</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="78.5" customHeight="1">
-      <x:c r="A9" s="47" t="s">
+      <x:c r="M9" s="46" t="s">
         <x:v>57</x:v>
-      </x:c>
-      <x:c r="B9" s="50" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="C9" s="47" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D9" s="47" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E9" s="47" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="F9" s="46" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="G9" s="47" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="H9" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="I9" s="47" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="J9" s="47" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="K9" s="46" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="L9" s="46" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="M9" s="46" t="s">
-        <x:v>64</x:v>
       </x:c>
       <x:c r="N9" s="47">
         <x:v>200</x:v>
@@ -2358,73 +2369,74 @@
       <x:c r="O9" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 405; message: This request method is not supported.</x:v>
       </x:c>
-      <x:c r="P9" s="47">
+      <x:c r="P9" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q9" s="46" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="R9" s="47">
+      <x:c r="Q9" s="46" t="str">
+        <x:v>200 transport | responseCode 405 | method not supported</x:v>
+      </x:c>
+      <x:c r="R9" s="47" t="n">
         <x:v>418</x:v>
       </x:c>
       <x:c r="S9" s="47" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="T9" s="47" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="U9" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V9" s="50" t="s">
-        <x:v>67</x:v>
+      <x:c r="T9" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U9" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V9" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-PRODUCT-002.png
+..\..\Automation\Execution Evidence\API-PRODUCT-002.png</x:v>
       </x:c>
       <x:c r="W9" s="51" t="str">
-        <x:v>NA</x:v>
-      </x:c>
-      <x:c r="X9" s="46" t="str">
-        <x:v>Validated contract: the transport status is HTTP 200 and the documented API code is JSON responseCode 405. The earlier defect was based on an incorrect status interpretation.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="78.5" customHeight="1">
+        <x:v>BUG-API-001</x:v>
+      </x:c>
+      <x:c r="X9" s="57" t="str">
+        <x:v>Current automated verification passed. The linked defect was rejected because the earlier failure came from request or assertion configuration, not product behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" s="47" t="s">
-        <x:v>68</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B10" s="50" t="s">
-        <x:v>69</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C10" s="47" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D10" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E10" s="47" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="E10" s="47" t="s">
-        <x:v>44</x:v>
-      </x:c>
       <x:c r="F10" s="46" t="s">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="G10" s="47" t="s">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="H10" s="47" t="s">
-        <x:v>71</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="I10" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J10" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="K10" s="46" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="L10" s="46" t="s">
-        <x:v>63</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="M10" s="46" t="s">
-        <x:v>72</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="N10" s="47">
         <x:v>200</x:v>
@@ -2432,73 +2444,74 @@
       <x:c r="O10" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 200; a non-empty brands array containing brand details.</x:v>
       </x:c>
-      <x:c r="P10" s="47">
+      <x:c r="P10" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q10" s="46" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="R10" s="47">
+      <x:c r="Q10" s="46" t="str">
+        <x:v>200 | brands list returned</x:v>
+      </x:c>
+      <x:c r="R10" s="47" t="n">
         <x:v>434</x:v>
       </x:c>
-      <x:c r="S10" s="47" t="s">
+      <x:c r="S10" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T10" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U10" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V10" s="55" t="str">
+        <x:v>..\Execution Results\Screenshots\API-BRAND-001.png
+..\..\Automation\Execution Evidence\API-BRAND-001.png</x:v>
+      </x:c>
+      <x:c r="W10" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X10" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="47" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B11" s="50" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="C11" s="47" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="T10" s="47" t="s">
+      <x:c r="E11" s="47" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="U10" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V10" s="52" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="W10" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="X10" s="46" t="s">
-        <x:v>75</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="78.5" customHeight="1">
-      <x:c r="A11" s="47" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="B11" s="50" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="C11" s="47" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D11" s="47" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E11" s="47" t="s">
-        <x:v>60</x:v>
-      </x:c>
       <x:c r="F11" s="46" t="s">
-        <x:v>78</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="G11" s="47" t="s">
-        <x:v>79</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="H11" s="47" t="s">
-        <x:v>71</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="I11" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J11" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="K11" s="46" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="L11" s="46" t="s">
-        <x:v>63</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="M11" s="46" t="s">
-        <x:v>80</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="N11" s="47">
         <x:v>200</x:v>
@@ -2506,73 +2519,74 @@
       <x:c r="O11" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 405; message: This request method is not supported.</x:v>
       </x:c>
-      <x:c r="P11" s="47">
+      <x:c r="P11" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q11" s="46" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="R11" s="47">
+      <x:c r="Q11" s="46" t="str">
+        <x:v>200 transport | responseCode 405 | method not supported</x:v>
+      </x:c>
+      <x:c r="R11" s="47" t="n">
         <x:v>468</x:v>
       </x:c>
-      <x:c r="S11" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="T11" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U11" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V11" s="50" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="W11" s="47" t="s">
+      <x:c r="S11" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T11" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U11" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V11" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-BRAND-002.png
+..\..\Automation\Execution Evidence\API-BRAND-002.png</x:v>
+      </x:c>
+      <x:c r="W11" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X11" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="47" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B12" s="50" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F12" s="46" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="G12" s="47" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="X11" s="46" t="s">
-        <x:v>83</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="78.5" customHeight="1">
-      <x:c r="A12" s="47" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="B12" s="50" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="C12" s="47" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D12" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E12" s="47" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F12" s="46" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="G12" s="47" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="H12" s="47" t="s">
-        <x:v>87</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I12" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J12" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K12" s="46" t="s">
-        <x:v>89</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="L12" s="46" t="s">
-        <x:v>63</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="M12" s="46" t="s">
-        <x:v>90</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="N12" s="47">
         <x:v>200</x:v>
@@ -2580,73 +2594,74 @@
       <x:c r="O12" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 200; a non-empty products array containing search results.</x:v>
       </x:c>
-      <x:c r="P12" s="47">
+      <x:c r="P12" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q12" s="46" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="R12" s="47">
+      <x:c r="Q12" s="46" t="str">
+        <x:v>200 | searched products list returned</x:v>
+      </x:c>
+      <x:c r="R12" s="47" t="n">
         <x:v>508</x:v>
       </x:c>
-      <x:c r="S12" s="47" t="s">
+      <x:c r="S12" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T12" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U12" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V12" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-SEARCH-001.png
+..\..\Automation\Execution Evidence\API-SEARCH-001.png</x:v>
+      </x:c>
+      <x:c r="W12" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X12" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58" customHeight="1">
+      <x:c r="A13" s="47" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B13" s="50" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="T12" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U12" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V12" s="50" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="W12" s="47" t="s">
+      <x:c r="E13" s="47" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F13" s="46" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G13" s="47" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="X12" s="46" t="s">
-        <x:v>93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="78.5" customHeight="1">
-      <x:c r="A13" s="47" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="B13" s="50" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="C13" s="47" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D13" s="47" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E13" s="47" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F13" s="46" t="s">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="G13" s="47" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="H13" s="47" t="s">
-        <x:v>87</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I13" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J13" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K13" s="46" t="s">
-        <x:v>97</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L13" s="46" t="s">
-        <x:v>63</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="M13" s="46" t="s">
-        <x:v>98</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="N13" s="47">
         <x:v>200</x:v>
@@ -2654,73 +2669,74 @@
       <x:c r="O13" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 400; message: Bad request, search_product parameter is missing in POST request.</x:v>
       </x:c>
-      <x:c r="P13" s="47">
+      <x:c r="P13" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q13" s="46" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="R13" s="47">
+      <x:c r="Q13" s="46" t="str">
+        <x:v>200 transport | responseCode 400 | missing search_product message returned</x:v>
+      </x:c>
+      <x:c r="R13" s="47" t="n">
         <x:v>406</x:v>
       </x:c>
       <x:c r="S13" s="47" t="str">
-        <x:v>Retest</x:v>
-      </x:c>
-      <x:c r="T13" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U13" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V13" s="53" t="s">
-        <x:v>100</x:v>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T13" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U13" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V13" s="56" t="str">
+        <x:v>..\Execution Results\Screenshots\API-SEARCH-002.png
+..\..\Automation\Execution Evidence\API-SEARCH-002.png</x:v>
       </x:c>
       <x:c r="W13" s="51" t="str">
-        <x:v>NA</x:v>
-      </x:c>
-      <x:c r="X13" s="46" t="str">
-        <x:v>Earlier Postman evidence used an incorrect request configuration. The automated request omitted search_product and returned the documented JSON responseCode 400. Clean rerun pending after the shared assertion fix.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="78.5" customHeight="1">
+        <x:v>BUG-API-002</x:v>
+      </x:c>
+      <x:c r="X13" s="57" t="str">
+        <x:v>Current automated verification passed. The linked defect was rejected because the earlier failure came from request or assertion configuration, not product behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" s="47" t="s">
-        <x:v>101</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B14" s="50" t="s">
-        <x:v>102</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C14" s="47" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="47" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E14" s="47" t="s">
-        <x:v>103</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F14" s="46" t="s">
-        <x:v>104</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="G14" s="47" t="s">
-        <x:v>62</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H14" s="47" t="s">
-        <x:v>105</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="I14" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J14" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K14" s="46" t="s">
-        <x:v>106</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="L14" s="46" t="s">
-        <x:v>107</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="M14" s="46" t="s">
-        <x:v>108</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="N14" s="47">
         <x:v>200</x:v>
@@ -2728,73 +2744,74 @@
       <x:c r="O14" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 200; message: User exists!</x:v>
       </x:c>
-      <x:c r="P14" s="47">
+      <x:c r="P14" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q14" s="46" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="R14" s="47">
+      <x:c r="Q14" s="46" t="str">
+        <x:v>200 transport | responseCode 200 | User exists!</x:v>
+      </x:c>
+      <x:c r="R14" s="47" t="n">
         <x:v>434</x:v>
       </x:c>
-      <x:c r="S14" s="47" t="s">
+      <x:c r="S14" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T14" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U14" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V14" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-AUTH-001.png
+..\..\Automation\Execution Evidence\API-AUTH-001.png</x:v>
+      </x:c>
+      <x:c r="W14" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X14" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="47" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B15" s="50" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="T14" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U14" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V14" s="50" t="s">
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="W14" s="47" t="s">
+      <x:c r="E15" s="47" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F15" s="46" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G15" s="47" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="X14" s="46" t="s">
-        <x:v>111</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="78.5" customHeight="1">
-      <x:c r="A15" s="47" t="s">
-        <x:v>112</x:v>
-      </x:c>
-      <x:c r="B15" s="50" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="C15" s="47" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D15" s="47" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E15" s="47" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F15" s="46" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="G15" s="47" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="H15" s="47" t="s">
-        <x:v>105</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="I15" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J15" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K15" s="46" t="s">
-        <x:v>115</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="L15" s="46" t="s">
-        <x:v>116</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="M15" s="46" t="s">
-        <x:v>117</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N15" s="47">
         <x:v>200</x:v>
@@ -2802,73 +2819,74 @@
       <x:c r="O15" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 400; message: Bad request, email or password parameter is missing in POST request.</x:v>
       </x:c>
-      <x:c r="P15" s="47">
+      <x:c r="P15" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q15" s="46" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="R15" s="47">
+      <x:c r="Q15" s="46" t="str">
+        <x:v>200 transport | responseCode 400 | missing credential message returned</x:v>
+      </x:c>
+      <x:c r="R15" s="47" t="n">
         <x:v>368</x:v>
       </x:c>
-      <x:c r="S15" s="47" t="s">
+      <x:c r="S15" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T15" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U15" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V15" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-AUTH-002.png
+..\..\Automation\Execution Evidence\API-AUTH-002.png</x:v>
+      </x:c>
+      <x:c r="W15" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X15" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="47" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B16" s="50" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="T15" s="47" t="s">
+      <x:c r="E16" s="47" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="U15" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V15" s="50" t="s">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="W15" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="X15" s="46" t="s">
-        <x:v>120</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="78.5" customHeight="1">
-      <x:c r="A16" s="47" t="s">
-        <x:v>121</x:v>
-      </x:c>
-      <x:c r="B16" s="50" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="C16" s="47" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D16" s="47" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E16" s="47" t="s">
-        <x:v>60</x:v>
-      </x:c>
       <x:c r="F16" s="46" t="s">
-        <x:v>123</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="G16" s="47" t="s">
-        <x:v>124</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="H16" s="47" t="s">
-        <x:v>105</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="I16" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J16" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="K16" s="46" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="L16" s="46" t="s">
-        <x:v>63</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="M16" s="46" t="s">
-        <x:v>125</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="N16" s="47">
         <x:v>200</x:v>
@@ -2876,73 +2894,74 @@
       <x:c r="O16" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 405; message: This request method is not supported.</x:v>
       </x:c>
-      <x:c r="P16" s="47">
+      <x:c r="P16" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q16" s="46" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="R16" s="47">
+      <x:c r="Q16" s="46" t="str">
+        <x:v>200 transport | responseCode 405 | method not supported</x:v>
+      </x:c>
+      <x:c r="R16" s="47" t="n">
         <x:v>423</x:v>
       </x:c>
-      <x:c r="S16" s="47" t="s">
+      <x:c r="S16" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T16" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U16" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V16" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-AUTH-003.png
+..\..\Automation\Execution Evidence\API-AUTH-003.png</x:v>
+      </x:c>
+      <x:c r="W16" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X16" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="47" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B17" s="50" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="T16" s="47" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="U16" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V16" s="50" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="W16" s="47" t="s">
+      <x:c r="E17" s="47" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F17" s="46" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="G17" s="47" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="X16" s="46" t="s">
-        <x:v>128</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="78.5" customHeight="1">
-      <x:c r="A17" s="47" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="B17" s="50" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="C17" s="47" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D17" s="47" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E17" s="47" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F17" s="46" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="G17" s="47" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="H17" s="47" t="s">
-        <x:v>105</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="I17" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J17" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K17" s="46" t="s">
-        <x:v>132</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="L17" s="46" t="s">
-        <x:v>133</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="M17" s="46" t="s">
-        <x:v>134</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="N17" s="47">
         <x:v>200</x:v>
@@ -2950,73 +2969,74 @@
       <x:c r="O17" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 404; message: User not found!</x:v>
       </x:c>
-      <x:c r="P17" s="47">
+      <x:c r="P17" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q17" s="46" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="R17" s="47">
+      <x:c r="Q17" s="46" t="str">
+        <x:v>200 transport | responseCode 404 | User not found!</x:v>
+      </x:c>
+      <x:c r="R17" s="47" t="n">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="S17" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="T17" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U17" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V17" s="50" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="W17" s="47" t="s">
+      <x:c r="S17" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T17" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U17" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V17" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-AUTH-004.png
+..\..\Automation\Execution Evidence\API-AUTH-004.png</x:v>
+      </x:c>
+      <x:c r="W17" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X17" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="58" customHeight="1">
+      <x:c r="A18" s="47" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B18" s="50" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C18" s="47" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="F18" s="46" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="G18" s="47" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="X17" s="46" t="s">
-        <x:v>137</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="78.5" customHeight="1">
-      <x:c r="A18" s="47" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="B18" s="50" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="C18" s="47" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D18" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E18" s="47" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="F18" s="46" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="G18" s="47" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="H18" s="47" t="s">
-        <x:v>141</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="I18" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J18" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K18" s="46" t="s">
-        <x:v>142</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="L18" s="46" t="s">
-        <x:v>143</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="M18" s="46" t="s">
-        <x:v>144</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="N18" s="47">
         <x:v>200</x:v>
@@ -3024,73 +3044,74 @@
       <x:c r="O18" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 201; message: User created!</x:v>
       </x:c>
-      <x:c r="P18" s="47">
+      <x:c r="P18" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q18" s="46" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="R18" s="47">
+      <x:c r="Q18" s="46" t="str">
+        <x:v>200 transport | responseCode 201 | User created!</x:v>
+      </x:c>
+      <x:c r="R18" s="47" t="n">
         <x:v>391</x:v>
       </x:c>
-      <x:c r="S18" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="T18" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U18" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V18" s="50" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="W18" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="X18" s="46" t="s">
-        <x:v>147</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="78.5" customHeight="1">
+      <x:c r="S18" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T18" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U18" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V18" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-001.png
+..\..\Automation\Execution Evidence\API-ACCOUNT-001.png</x:v>
+      </x:c>
+      <x:c r="W18" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X18" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" s="47" t="s">
-        <x:v>148</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B19" s="50" t="s">
-        <x:v>149</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C19" s="47" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D19" s="47" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E19" s="47" t="s">
-        <x:v>103</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F19" s="46" t="s">
-        <x:v>150</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="G19" s="47" t="s">
-        <x:v>124</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="H19" s="47" t="s">
-        <x:v>151</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="I19" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J19" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K19" s="46" t="s">
-        <x:v>152</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="L19" s="46" t="s">
-        <x:v>153</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="M19" s="46" t="s">
-        <x:v>154</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="N19" s="47">
         <x:v>200</x:v>
@@ -3098,73 +3119,74 @@
       <x:c r="O19" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 200; message: Account deleted!</x:v>
       </x:c>
-      <x:c r="P19" s="47">
+      <x:c r="P19" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q19" s="46" t="s">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="R19" s="47">
+      <x:c r="Q19" s="46" t="str">
+        <x:v>200 transport | responseCode 200 | Account deleted!</x:v>
+      </x:c>
+      <x:c r="R19" s="47" t="n">
         <x:v>481</x:v>
       </x:c>
-      <x:c r="S19" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="T19" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U19" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V19" s="50" t="s">
-        <x:v>156</x:v>
-      </x:c>
-      <x:c r="W19" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="X19" s="46" t="s">
-        <x:v>157</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="78.5" customHeight="1">
+      <x:c r="S19" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T19" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U19" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V19" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-002.png
+..\..\Automation\Execution Evidence\API-ACCOUNT-002.png</x:v>
+      </x:c>
+      <x:c r="W19" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X19" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" s="47" t="s">
-        <x:v>158</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B20" s="50" t="s">
-        <x:v>159</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C20" s="47" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D20" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E20" s="47" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="E20" s="47" t="s">
-        <x:v>44</x:v>
-      </x:c>
       <x:c r="F20" s="46" t="s">
-        <x:v>160</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="G20" s="47" t="s">
-        <x:v>79</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="H20" s="47" t="s">
-        <x:v>161</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="I20" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J20" s="47" t="s">
-        <x:v>88</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K20" s="46" t="s">
-        <x:v>162</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="L20" s="46" t="s">
-        <x:v>153</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="M20" s="46" t="s">
-        <x:v>163</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="N20" s="47">
         <x:v>200</x:v>
@@ -3172,73 +3194,74 @@
       <x:c r="O20" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 200; message: User updated!</x:v>
       </x:c>
-      <x:c r="P20" s="47">
+      <x:c r="P20" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q20" s="46" t="s">
-        <x:v>164</x:v>
-      </x:c>
-      <x:c r="R20" s="47">
+      <x:c r="Q20" s="46" t="str">
+        <x:v>200 transport | responseCode 200 | User updated!</x:v>
+      </x:c>
+      <x:c r="R20" s="47" t="n">
         <x:v>379</x:v>
       </x:c>
-      <x:c r="S20" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="T20" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U20" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V20" s="50" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="W20" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="X20" s="46" t="s">
+      <x:c r="S20" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T20" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U20" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V20" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-003.png
+..\..\Automation\Execution Evidence\API-ACCOUNT-003.png</x:v>
+      </x:c>
+      <x:c r="W20" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X20" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="58" customHeight="1">
+      <x:c r="A21" s="47" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="B21" s="50" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C21" s="47" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E21" s="47" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F21" s="46" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="G21" s="47" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="H21" s="47" t="s">
         <x:v>128</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="78.5" customHeight="1">
-      <x:c r="A21" s="47" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="B21" s="50" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="C21" s="47" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D21" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E21" s="47" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F21" s="46" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="G21" s="47" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="H21" s="47" t="s">
-        <x:v>169</x:v>
-      </x:c>
       <x:c r="I21" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J21" s="47" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="K21" s="46" t="s">
-        <x:v>170</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="L21" s="46" t="s">
-        <x:v>171</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="M21" s="46" t="s">
-        <x:v>172</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="N21" s="47">
         <x:v>200</x:v>
@@ -3246,32 +3269,33 @@
       <x:c r="O21" s="46" t="str">
         <x:v>HTTP 200; JSON responseCode 200; User Detail JSON for the requested email.</x:v>
       </x:c>
-      <x:c r="P21" s="47">
+      <x:c r="P21" s="47" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="Q21" s="46" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="R21" s="47">
+      <x:c r="Q21" s="46" t="str">
+        <x:v>200 transport | responseCode 200 | user detail returned</x:v>
+      </x:c>
+      <x:c r="R21" s="47" t="n">
         <x:v>358</x:v>
       </x:c>
-      <x:c r="S21" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="T21" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="U21" s="49">
-        <x:v>46235</x:v>
-      </x:c>
-      <x:c r="V21" s="50" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="W21" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="X21" s="46" t="s">
-        <x:v>175</x:v>
+      <x:c r="S21" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="T21" s="47" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="U21" s="49" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V21" s="54" t="str">
+        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-004.png
+..\..\Automation\Execution Evidence\API-ACCOUNT-004.png</x:v>
+      </x:c>
+      <x:c r="W21" s="47" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="X21" s="57" t="str">
+        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3294,7 +3318,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R734b583c60de4ec5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4830e1dfce18425c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3312,7 +3336,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="11" t="s">
-        <x:v>176</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B1" s="11"/>
       <x:c r="C1" s="11"/>
@@ -3324,7 +3348,7 @@
     </x:row>
     <x:row r="3" ht="15.5">
       <x:c r="A3" s="44" t="s">
-        <x:v>177</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B3" s="44"/>
       <x:c r="C3" s="44"/>
@@ -3404,83 +3428,83 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5" t="s">
-        <x:v>178</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
-        <x:v>179</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C11" s="6" t="s">
-        <x:v>180</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D11" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="47" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B12" s="47" t="s">
-        <x:v>182</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C12" s="47" t="s">
-        <x:v>183</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D12" s="47" t="s">
-        <x:v>184</x:v>
+        <x:v>140</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="47" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B13" s="47" t="s">
-        <x:v>182</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C13" s="47" t="s">
-        <x:v>185</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D13" s="47" t="s">
-        <x:v>186</x:v>
+        <x:v>142</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="47" t="s">
-        <x:v>187</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B14" s="47" t="s">
-        <x:v>182</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C14" s="47" t="s">
-        <x:v>188</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="D14" s="47" t="s">
-        <x:v>189</x:v>
+        <x:v>145</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="47" t="s">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B15" s="47" t="s">
-        <x:v>190</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="C15" s="47" t="s">
-        <x:v>191</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="D15" s="47" t="s">
-        <x:v>192</x:v>
+        <x:v>148</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="47" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B16" s="47" t="s">
-        <x:v>182</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C16" s="47" t="s">
-        <x:v>193</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="D16" s="47" t="str">
         <x:v>Use HTTP 200 for this application. Record the official scenario code inside Expected Response as the JSON responseCode.</x:v>
@@ -3488,100 +3512,100 @@
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="47" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B17" s="47" t="s">
-        <x:v>194</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C17" s="47" t="s">
-        <x:v>195</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D17" s="47" t="s">
-        <x:v>196</x:v>
+        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="47" t="s">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B18" s="47" t="s">
-        <x:v>194</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C18" s="47" t="s">
-        <x:v>197</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D18" s="47" t="s">
-        <x:v>198</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="47" t="s">
-        <x:v>199</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B19" s="47" t="s">
-        <x:v>194</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C19" s="47" t="s">
-        <x:v>200</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D19" s="47" t="s">
-        <x:v>201</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="47" t="s">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B20" s="47" t="s">
-        <x:v>182</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C20" s="47" t="s">
-        <x:v>202</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="D20" s="47" t="s">
-        <x:v>203</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="47" t="s">
-        <x:v>204</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B21" s="47" t="s">
-        <x:v>194</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C21" s="47" t="s">
-        <x:v>205</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="D21" s="47" t="s">
-        <x:v>206</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="47" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B22" s="47" t="s">
-        <x:v>207</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C22" s="47" t="s">
-        <x:v>208</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D22" s="47" t="s">
-        <x:v>209</x:v>
+        <x:v>165</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="47" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B23" s="47" t="s">
-        <x:v>210</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="C23" s="47" t="s">
-        <x:v>211</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D23" s="47" t="s">
-        <x:v>212</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3607,97 +3631,445 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="8" t="s">
-        <x:v>213</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B1" s="9" t="s">
-        <x:v>214</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C1" s="9" t="s">
-        <x:v>215</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="D1" s="9" t="s">
-        <x:v>216</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="E1" s="10" t="s">
-        <x:v>217</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="48" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="48" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C2" s="48" t="s">
-        <x:v>103</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D2" s="48" t="s">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E2" s="48" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="48" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B3" s="48" t="s">
-        <x:v>59</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C3" s="48" t="s">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D3" s="48" t="s">
-        <x:v>62</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E3" s="48" t="s">
-        <x:v>52</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="48" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B4" s="48"/>
       <x:c r="C4" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D4" s="48" t="s">
-        <x:v>79</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E4" s="48" t="s">
-        <x:v>218</x:v>
+        <x:v>175</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="48" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B5" s="48"/>
       <x:c r="C5" s="48" t="s">
-        <x:v>219</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D5" s="48" t="s">
-        <x:v>124</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="E5" s="48" t="s">
-        <x:v>220</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="48" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B6" s="48"/>
       <x:c r="C6" s="48"/>
       <x:c r="D6" s="48"/>
       <x:c r="E6" s="48" t="s">
-        <x:v>221</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="76" t="str">
+        <x:v>Automation Exercise | API Execution Summary</x:v>
+      </x:c>
+      <x:c r="B1" s="76"/>
+      <x:c r="C1" s="76"/>
+      <x:c r="D1" s="76"/>
+      <x:c r="E1" s="76"/>
+      <x:c r="F1" s="76"/>
+      <x:c r="G1" s="76"/>
+      <x:c r="H1" s="76"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="77" t="str">
+        <x:v>Reconciled 2026-08-09 | authoritative requirements, Postman baseline, current verification, evidence, and defect disposition</x:v>
+      </x:c>
+      <x:c r="B2" s="77"/>
+      <x:c r="C2" s="77"/>
+      <x:c r="D2" s="77"/>
+      <x:c r="E2" s="77"/>
+      <x:c r="F2" s="77"/>
+      <x:c r="G2" s="77"/>
+      <x:c r="H2" s="77"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="78"/>
+      <x:c r="B3" s="78"/>
+      <x:c r="C3" s="78"/>
+      <x:c r="D3" s="78"/>
+      <x:c r="E3" s="78"/>
+      <x:c r="F3" s="78"/>
+      <x:c r="G3" s="78"/>
+      <x:c r="H3" s="78"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="78" t="str">
+        <x:v>Current requirement result</x:v>
+      </x:c>
+      <x:c r="B4" s="78" t="str">
+        <x:v>14 Passed | 0 Failed | 0 Not Run</x:v>
+      </x:c>
+      <x:c r="C4" s="78"/>
+      <x:c r="D4" s="78"/>
+      <x:c r="E4" s="78"/>
+      <x:c r="F4" s="79" t="str">
+        <x:v>Evidence source</x:v>
+      </x:c>
+      <x:c r="G4" s="79" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="H4" s="79" t="str">
+        <x:v>Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="78" t="str">
+        <x:v>Historical Postman baseline</x:v>
+      </x:c>
+      <x:c r="B5" s="78" t="str">
+        <x:v>37 assertions | 28 passed | 9 failed | 2 runner errors</x:v>
+      </x:c>
+      <x:c r="C5" s="78"/>
+      <x:c r="D5" s="78"/>
+      <x:c r="E5" s="78"/>
+      <x:c r="F5" s="78" t="str">
+        <x:v>Postman runner</x:v>
+      </x:c>
+      <x:c r="G5" s="78" t="str">
+        <x:v>Historical execution baseline</x:v>
+      </x:c>
+      <x:c r="H5" s="78" t="str">
+        <x:v>Execution Results\Postman Reports</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="78" t="str">
+        <x:v>Current automated verification</x:v>
+      </x:c>
+      <x:c r="B6" s="78" t="str">
+        <x:v>14 of 14 canonical API scenarios passed</x:v>
+      </x:c>
+      <x:c r="C6" s="78"/>
+      <x:c r="D6" s="78"/>
+      <x:c r="E6" s="78"/>
+      <x:c r="F6" s="78" t="str">
+        <x:v>Postman screenshots</x:v>
+      </x:c>
+      <x:c r="G6" s="78" t="str">
+        <x:v>Request and response evidence</x:v>
+      </x:c>
+      <x:c r="H6" s="78" t="str">
+        <x:v>Execution Results\Screenshots</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="78" t="str">
+        <x:v>Open confirmed API defects</x:v>
+      </x:c>
+      <x:c r="B7" s="78" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="78"/>
+      <x:c r="D7" s="78"/>
+      <x:c r="E7" s="78"/>
+      <x:c r="F7" s="78" t="str">
+        <x:v>Playwright API validation</x:v>
+      </x:c>
+      <x:c r="G7" s="78" t="str">
+        <x:v>Current independent verification</x:v>
+      </x:c>
+      <x:c r="H7" s="78" t="str">
+        <x:v>..\..\Automation\Execution Evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="78" t="str">
+        <x:v>Rejected configuration defects</x:v>
+      </x:c>
+      <x:c r="B8" s="78" t="str">
+        <x:v>BUG-API-001 | BUG-API-002</x:v>
+      </x:c>
+      <x:c r="C8" s="78"/>
+      <x:c r="D8" s="78"/>
+      <x:c r="E8" s="78"/>
+      <x:c r="F8" s="78"/>
+      <x:c r="G8" s="78"/>
+      <x:c r="H8" s="78"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="78"/>
+      <x:c r="B9" s="78"/>
+      <x:c r="C9" s="78"/>
+      <x:c r="D9" s="78"/>
+      <x:c r="E9" s="78"/>
+      <x:c r="F9" s="78"/>
+      <x:c r="G9" s="78"/>
+      <x:c r="H9" s="78"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="79" t="str">
+        <x:v>Module</x:v>
+      </x:c>
+      <x:c r="B10" s="79" t="str">
+        <x:v>Requirements</x:v>
+      </x:c>
+      <x:c r="C10" s="79" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="D10" s="79" t="str">
+        <x:v>Coverage</x:v>
+      </x:c>
+      <x:c r="E10" s="78"/>
+      <x:c r="F10" s="78"/>
+      <x:c r="G10" s="78"/>
+      <x:c r="H10" s="78"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="78" t="str">
+        <x:v>Products</x:v>
+      </x:c>
+      <x:c r="B11" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C11" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D11" s="78" t="str">
+        <x:v>100%</x:v>
+      </x:c>
+      <x:c r="E11" s="78"/>
+      <x:c r="F11" s="78"/>
+      <x:c r="G11" s="78"/>
+      <x:c r="H11" s="78"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="78" t="str">
+        <x:v>Brands</x:v>
+      </x:c>
+      <x:c r="B12" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C12" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D12" s="78" t="str">
+        <x:v>100%</x:v>
+      </x:c>
+      <x:c r="E12" s="78"/>
+      <x:c r="F12" s="78"/>
+      <x:c r="G12" s="78"/>
+      <x:c r="H12" s="78"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="78" t="str">
+        <x:v>Product Search</x:v>
+      </x:c>
+      <x:c r="B13" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C13" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D13" s="78" t="str">
+        <x:v>100%</x:v>
+      </x:c>
+      <x:c r="E13" s="78"/>
+      <x:c r="F13" s="78"/>
+      <x:c r="G13" s="78"/>
+      <x:c r="H13" s="78"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="78" t="str">
+        <x:v>Authentication</x:v>
+      </x:c>
+      <x:c r="B14" s="78" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C14" s="78" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D14" s="78" t="str">
+        <x:v>100%</x:v>
+      </x:c>
+      <x:c r="E14" s="78"/>
+      <x:c r="F14" s="78"/>
+      <x:c r="G14" s="78"/>
+      <x:c r="H14" s="78"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="78" t="str">
+        <x:v>Account Management</x:v>
+      </x:c>
+      <x:c r="B15" s="78" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C15" s="78" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D15" s="78" t="str">
+        <x:v>100%</x:v>
+      </x:c>
+      <x:c r="E15" s="78"/>
+      <x:c r="F15" s="78"/>
+      <x:c r="G15" s="78"/>
+      <x:c r="H15" s="78"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="78"/>
+      <x:c r="B16" s="78"/>
+      <x:c r="C16" s="78"/>
+      <x:c r="D16" s="78"/>
+      <x:c r="E16" s="78"/>
+      <x:c r="F16" s="78"/>
+      <x:c r="G16" s="78"/>
+      <x:c r="H16" s="78"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="80" t="str">
+        <x:v>Interpretation note</x:v>
+      </x:c>
+      <x:c r="B17" s="80"/>
+      <x:c r="C17" s="80"/>
+      <x:c r="D17" s="80"/>
+      <x:c r="E17" s="80"/>
+      <x:c r="F17" s="80"/>
+      <x:c r="G17" s="80"/>
+      <x:c r="H17" s="80"/>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" s="81" t="str">
+        <x:v>Automation Exercise returns HTTP transport status 200 for these endpoints and places the documented business result in the JSON responseCode field. The historical Postman failures were retained for auditability, then reconciled against the official API specification and current automated evidence. They do not represent nine confirmed product defects.</x:v>
+      </x:c>
+      <x:c r="B18" s="81"/>
+      <x:c r="C18" s="81"/>
+      <x:c r="D18" s="81"/>
+      <x:c r="E18" s="81"/>
+      <x:c r="F18" s="81"/>
+      <x:c r="G18" s="81"/>
+      <x:c r="H18" s="81"/>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="81"/>
+      <x:c r="B19" s="81"/>
+      <x:c r="C19" s="81"/>
+      <x:c r="D19" s="81"/>
+      <x:c r="E19" s="81"/>
+      <x:c r="F19" s="81"/>
+      <x:c r="G19" s="81"/>
+      <x:c r="H19" s="81"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="81"/>
+      <x:c r="B20" s="81"/>
+      <x:c r="C20" s="81"/>
+      <x:c r="D20" s="81"/>
+      <x:c r="E20" s="81"/>
+      <x:c r="F20" s="81"/>
+      <x:c r="G20" s="81"/>
+      <x:c r="H20" s="81"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="78"/>
+      <x:c r="B21" s="78"/>
+      <x:c r="C21" s="78"/>
+      <x:c r="D21" s="78"/>
+      <x:c r="E21" s="78"/>
+      <x:c r="F21" s="78"/>
+      <x:c r="G21" s="78"/>
+      <x:c r="H21" s="78"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="82" t="str">
+        <x:v>QA sign-off | all 14 official API requirements are traceable, executed, evidenced, and currently passing. The Postman collection should be rerun after assertion updates whenever the service changes.</x:v>
+      </x:c>
+      <x:c r="B22" s="82"/>
+      <x:c r="C22" s="82"/>
+      <x:c r="D22" s="82"/>
+      <x:c r="E22" s="82"/>
+      <x:c r="F22" s="82"/>
+      <x:c r="G22" s="82"/>
+      <x:c r="H22" s="82"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A17:H17"/>
+    <x:mergeCell ref="A18:H20"/>
+    <x:mergeCell ref="A22:H22"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
artifact audit and sync
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/API Testing/Documentation/Automation Exercise API Test Cases.xlsx
+++ b/Automation Exercise Project/API Testing/Documentation/Automation Exercise API Test Cases.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Raa6bd72c3b12435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Test Cases" sheetId="2" r:id="R3aa19c111ecd4857"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="Re5a15a69522645c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R6aaf1d6907b249b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Summary" sheetId="5" r:id="R22bd8e4fb33f4b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra068fe473d484525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Test Cases" sheetId="2" r:id="Racbf0e98ca4d4419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R27961b58190440a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R1863b52dad494ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Summary" sheetId="5" r:id="Rff60f87b119d43fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,9 +42,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Products</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Execute one request at a time in Postman. Record the observed HTTP status, response body summary, response time, status, executor, date, and evidence path. If a result fails, create a defect and enter its ID. Never place real passwords, tokens, or personal data in this workbook or screenshots.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Brands</x:t>
@@ -1784,7 +1781,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>Professional API QA repository | 14 official requirements | historical Postman baseline plus current automated verification</x:v>
+        <x:v>Professional API QA repository | 14 official requirements | clean Postman run plus independent Playwright verification</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -1900,8 +1897,8 @@
         <x:f>B9-C9</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F9" s="23" t="s">
-        <x:v>10</x:v>
+      <x:c r="F9" s="23" t="str">
+        <x:v>Latest controlled execution: the corrected 14-request Postman collection ran once on 2026-08-09 and passed 42 of 42 assertions with zero errors. Record transport status, JSON responseCode, payload/message result, duration, evidence, and defect disposition separately. Never publish credentials or personal test data.</x:v>
       </x:c>
       <x:c r="G9" s="24"/>
       <x:c r="H9" s="24"/>
@@ -1914,7 +1911,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="45" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B10" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A10)</x:f>
@@ -1940,7 +1937,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="45" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B11" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A11)</x:f>
@@ -1966,7 +1963,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B12" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A12)</x:f>
@@ -1992,7 +1989,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B13" s="45" t="n">
         <x:f>COUNTIF('API Test Cases'!C8:C21,A13)</x:f>
@@ -2066,7 +2063,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="11" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B1" s="11"/>
       <x:c r="C1" s="11"/>
@@ -2122,7 +2119,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="32" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="33"/>
       <x:c r="C4" s="33"/>
@@ -2132,7 +2129,7 @@
       <x:c r="G4" s="33"/>
       <x:c r="H4" s="34"/>
       <x:c r="J4" s="38" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="K4" s="39"/>
       <x:c r="L4" s="39"/>
@@ -2176,117 +2173,117 @@
     </x:row>
     <x:row r="7" ht="44" customHeight="1">
       <x:c r="A7" s="4" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="s">
         <x:v>18</x:v>
-      </x:c>
-      <x:c r="B7" s="4" t="s">
-        <x:v>19</x:v>
       </x:c>
       <x:c r="C7" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="E7" s="4" t="s">
+      <x:c r="F7" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="s">
+      <x:c r="G7" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="G7" s="4" t="s">
+      <x:c r="H7" s="4" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="H7" s="4" t="s">
+      <x:c r="I7" s="4" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="I7" s="4" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="J7" s="4" t="s">
+      <x:c r="K7" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="K7" s="4" t="s">
+      <x:c r="L7" s="4" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L7" s="4" t="s">
+      <x:c r="M7" s="4" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="M7" s="4" t="s">
+      <x:c r="N7" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="N7" s="4" t="s">
+      <x:c r="O7" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="O7" s="4" t="s">
+      <x:c r="P7" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="P7" s="4" t="s">
+      <x:c r="Q7" s="4" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="Q7" s="4" t="s">
+      <x:c r="R7" s="4" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="R7" s="4" t="s">
+      <x:c r="S7" s="4" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="S7" s="4" t="s">
+      <x:c r="T7" s="4" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="T7" s="4" t="s">
+      <x:c r="U7" s="4" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="U7" s="4" t="s">
+      <x:c r="V7" s="4" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="V7" s="4" t="s">
+      <x:c r="W7" s="4" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="W7" s="4" t="s">
+      <x:c r="X7" s="4" t="s">
         <x:v>38</x:v>
-      </x:c>
-      <x:c r="X7" s="4" t="s">
-        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="47" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B8" s="50" t="s">
         <x:v>40</x:v>
-      </x:c>
-      <x:c r="B8" s="50" t="s">
-        <x:v>41</x:v>
       </x:c>
       <x:c r="C8" s="47" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D8" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="E8" s="47" t="s">
+      <x:c r="F8" s="46" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="F8" s="46" t="s">
+      <x:c r="G8" s="47" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="G8" s="47" t="s">
+      <x:c r="H8" s="47" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="H8" s="47" t="s">
+      <x:c r="I8" s="47" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="I8" s="47" t="s">
+      <x:c r="J8" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="K8" s="46" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="L8" s="46" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="J8" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="K8" s="46" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="L8" s="46" t="s">
+      <x:c r="M8" s="46" t="s">
         <x:v>48</x:v>
-      </x:c>
-      <x:c r="M8" s="46" t="s">
-        <x:v>49</x:v>
       </x:c>
       <x:c r="N8" s="47">
         <x:v>200</x:v>
@@ -2301,7 +2298,7 @@
         <x:v>200 | products list returned</x:v>
       </x:c>
       <x:c r="R8" s="47" t="n">
-        <x:v>616</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="S8" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2310,58 +2307,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U8" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V8" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-PRODUCT-001.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-PRODUCT-001.png
 ..\..\Automation\Execution Evidence\API-PRODUCT-001.png</x:v>
       </x:c>
       <x:c r="W8" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X8" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="47" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B9" s="50" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="B9" s="50" t="s">
-        <x:v>51</x:v>
       </x:c>
       <x:c r="C9" s="47" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D9" s="47" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="E9" s="47" t="s">
+      <x:c r="F9" s="46" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="F9" s="46" t="s">
+      <x:c r="G9" s="47" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G9" s="47" t="s">
+      <x:c r="H9" s="47" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="I9" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J9" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="K9" s="46" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="L9" s="46" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="H9" s="47" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="I9" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J9" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="K9" s="46" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="L9" s="46" t="s">
+      <x:c r="M9" s="46" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="M9" s="46" t="s">
-        <x:v>57</x:v>
       </x:c>
       <x:c r="N9" s="47">
         <x:v>200</x:v>
@@ -2376,7 +2375,7 @@
         <x:v>200 transport | responseCode 405 | method not supported</x:v>
       </x:c>
       <x:c r="R9" s="47" t="n">
-        <x:v>418</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="S9" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2385,58 +2384,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U9" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V9" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-PRODUCT-002.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-PRODUCT-002.png
 ..\..\Automation\Execution Evidence\API-PRODUCT-002.png</x:v>
       </x:c>
       <x:c r="W9" s="51" t="str">
         <x:v>BUG-API-001</x:v>
       </x:c>
       <x:c r="X9" s="57" t="str">
-        <x:v>Current automated verification passed. The linked defect was rejected because the earlier failure came from request or assertion configuration, not product behavior.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" s="47" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B10" s="50" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B10" s="50" t="s">
+      <x:c r="C10" s="47" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D10" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E10" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F10" s="46" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="C10" s="47" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D10" s="47" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E10" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F10" s="46" t="s">
+      <x:c r="G10" s="47" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="H10" s="47" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G10" s="47" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="H10" s="47" t="s">
+      <x:c r="I10" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J10" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="K10" s="46" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="L10" s="46" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="M10" s="46" t="s">
         <x:v>61</x:v>
-      </x:c>
-      <x:c r="I10" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J10" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="K10" s="46" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="L10" s="46" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="M10" s="46" t="s">
-        <x:v>62</x:v>
       </x:c>
       <x:c r="N10" s="47">
         <x:v>200</x:v>
@@ -2451,7 +2452,7 @@
         <x:v>200 | brands list returned</x:v>
       </x:c>
       <x:c r="R10" s="47" t="n">
-        <x:v>434</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="S10" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2460,58 +2461,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U10" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V10" s="55" t="str">
-        <x:v>..\Execution Results\Screenshots\API-BRAND-001.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-BRAND-001.png
 ..\..\Automation\Execution Evidence\API-BRAND-001.png</x:v>
       </x:c>
       <x:c r="W10" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X10" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" s="47" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B11" s="50" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="B11" s="50" t="s">
+      <x:c r="C11" s="47" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E11" s="47" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F11" s="46" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="C11" s="47" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D11" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="E11" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="F11" s="46" t="s">
+      <x:c r="G11" s="47" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="G11" s="47" t="s">
+      <x:c r="H11" s="47" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="I11" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J11" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="K11" s="46" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="L11" s="46" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="M11" s="46" t="s">
         <x:v>66</x:v>
-      </x:c>
-      <x:c r="H11" s="47" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I11" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J11" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="K11" s="46" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="L11" s="46" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="M11" s="46" t="s">
-        <x:v>67</x:v>
       </x:c>
       <x:c r="N11" s="47">
         <x:v>200</x:v>
@@ -2526,7 +2529,7 @@
         <x:v>200 transport | responseCode 405 | method not supported</x:v>
       </x:c>
       <x:c r="R11" s="47" t="n">
-        <x:v>468</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="S11" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2535,58 +2538,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U11" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V11" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-BRAND-002.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-BRAND-002.png
 ..\..\Automation\Execution Evidence\API-BRAND-002.png</x:v>
       </x:c>
       <x:c r="W11" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X11" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" s="47" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B12" s="50" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B12" s="50" t="s">
+      <x:c r="C12" s="47" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F12" s="46" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C12" s="47" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D12" s="47" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E12" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F12" s="46" t="s">
+      <x:c r="G12" s="47" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H12" s="47" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="G12" s="47" t="s">
+      <x:c r="I12" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J12" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K12" s="46" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="L12" s="46" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="H12" s="47" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="I12" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J12" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K12" s="46" t="s">
+      <x:c r="M12" s="46" t="s">
         <x:v>73</x:v>
-      </x:c>
-      <x:c r="L12" s="46" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="M12" s="46" t="s">
-        <x:v>74</x:v>
       </x:c>
       <x:c r="N12" s="47">
         <x:v>200</x:v>
@@ -2601,7 +2606,7 @@
         <x:v>200 | searched products list returned</x:v>
       </x:c>
       <x:c r="R12" s="47" t="n">
-        <x:v>508</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="S12" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2610,58 +2615,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U12" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V12" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-SEARCH-001.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-SEARCH-001.png
 ..\..\Automation\Execution Evidence\API-SEARCH-001.png</x:v>
       </x:c>
       <x:c r="W12" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X12" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" s="47" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B13" s="50" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B13" s="50" t="s">
+      <x:c r="C13" s="47" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F13" s="46" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="C13" s="47" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D13" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="E13" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F13" s="46" t="s">
+      <x:c r="G13" s="47" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H13" s="47" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="I13" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J13" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K13" s="46" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="G13" s="47" t="s">
+      <x:c r="L13" s="46" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="H13" s="47" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="I13" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J13" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K13" s="46" t="s">
+      <x:c r="M13" s="46" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="L13" s="46" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="M13" s="46" t="s">
-        <x:v>79</x:v>
       </x:c>
       <x:c r="N13" s="47">
         <x:v>200</x:v>
@@ -2676,7 +2683,7 @@
         <x:v>200 transport | responseCode 400 | missing search_product message returned</x:v>
       </x:c>
       <x:c r="R13" s="47" t="n">
-        <x:v>406</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="S13" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2685,58 +2692,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U13" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V13" s="56" t="str">
-        <x:v>..\Execution Results\Screenshots\API-SEARCH-002.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-SEARCH-002.png
 ..\..\Automation\Execution Evidence\API-SEARCH-002.png</x:v>
       </x:c>
       <x:c r="W13" s="51" t="str">
         <x:v>BUG-API-002</x:v>
       </x:c>
       <x:c r="X13" s="57" t="str">
-        <x:v>Current automated verification passed. The linked defect was rejected because the earlier failure came from request or assertion configuration, not product behavior.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" s="47" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="B14" s="50" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="B14" s="50" t="s">
+      <x:c r="C14" s="47" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="C14" s="47" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D14" s="47" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E14" s="47" t="s">
+      <x:c r="F14" s="46" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="F14" s="46" t="s">
+      <x:c r="G14" s="47" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H14" s="47" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="G14" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="H14" s="47" t="s">
+      <x:c r="I14" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J14" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K14" s="46" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="I14" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J14" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K14" s="46" t="s">
+      <x:c r="L14" s="46" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="L14" s="46" t="s">
+      <x:c r="M14" s="46" t="s">
         <x:v>86</x:v>
-      </x:c>
-      <x:c r="M14" s="46" t="s">
-        <x:v>87</x:v>
       </x:c>
       <x:c r="N14" s="47">
         <x:v>200</x:v>
@@ -2751,7 +2760,7 @@
         <x:v>200 transport | responseCode 200 | User exists!</x:v>
       </x:c>
       <x:c r="R14" s="47" t="n">
-        <x:v>434</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="S14" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2760,58 +2769,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U14" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V14" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-AUTH-001.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-AUTH-001.png
 ..\..\Automation\Execution Evidence\API-AUTH-001.png</x:v>
       </x:c>
       <x:c r="W14" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X14" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="47" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B15" s="50" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B15" s="50" t="s">
+      <x:c r="C15" s="47" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F15" s="46" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="C15" s="47" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D15" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="E15" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F15" s="46" t="s">
+      <x:c r="G15" s="47" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H15" s="47" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="I15" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J15" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K15" s="46" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="G15" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="H15" s="47" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="I15" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J15" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K15" s="46" t="s">
+      <x:c r="L15" s="46" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="L15" s="46" t="s">
+      <x:c r="M15" s="46" t="s">
         <x:v>92</x:v>
-      </x:c>
-      <x:c r="M15" s="46" t="s">
-        <x:v>93</x:v>
       </x:c>
       <x:c r="N15" s="47">
         <x:v>200</x:v>
@@ -2826,7 +2837,7 @@
         <x:v>200 transport | responseCode 400 | missing credential message returned</x:v>
       </x:c>
       <x:c r="R15" s="47" t="n">
-        <x:v>368</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="S15" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2835,58 +2846,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U15" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V15" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-AUTH-002.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-AUTH-002.png
 ..\..\Automation\Execution Evidence\API-AUTH-002.png</x:v>
       </x:c>
       <x:c r="W15" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X15" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" s="47" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B16" s="50" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="B16" s="50" t="s">
+      <x:c r="C16" s="47" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F16" s="46" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="C16" s="47" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D16" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="E16" s="47" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="F16" s="46" t="s">
+      <x:c r="G16" s="47" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="G16" s="47" t="s">
+      <x:c r="H16" s="47" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="I16" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J16" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="K16" s="46" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="L16" s="46" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="M16" s="46" t="s">
         <x:v>97</x:v>
-      </x:c>
-      <x:c r="H16" s="47" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="I16" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J16" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="K16" s="46" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="L16" s="46" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="M16" s="46" t="s">
-        <x:v>98</x:v>
       </x:c>
       <x:c r="N16" s="47">
         <x:v>200</x:v>
@@ -2901,7 +2914,7 @@
         <x:v>200 transport | responseCode 405 | method not supported</x:v>
       </x:c>
       <x:c r="R16" s="47" t="n">
-        <x:v>423</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="S16" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2910,58 +2923,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U16" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V16" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-AUTH-003.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-AUTH-003.png
 ..\..\Automation\Execution Evidence\API-AUTH-003.png</x:v>
       </x:c>
       <x:c r="W16" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X16" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" s="47" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B17" s="50" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="B17" s="50" t="s">
+      <x:c r="C17" s="47" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F17" s="46" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C17" s="47" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D17" s="47" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="E17" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F17" s="46" t="s">
+      <x:c r="G17" s="47" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H17" s="47" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="I17" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J17" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K17" s="46" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="G17" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="H17" s="47" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="I17" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J17" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K17" s="46" t="s">
+      <x:c r="L17" s="46" t="s">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="L17" s="46" t="s">
+      <x:c r="M17" s="46" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="M17" s="46" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="N17" s="47">
         <x:v>200</x:v>
@@ -2976,7 +2991,7 @@
         <x:v>200 transport | responseCode 404 | User not found!</x:v>
       </x:c>
       <x:c r="R17" s="47" t="n">
-        <x:v>127</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="S17" s="47" t="str">
         <x:v>Pass</x:v>
@@ -2985,58 +3000,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U17" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V17" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-AUTH-004.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-AUTH-004.png
 ..\..\Automation\Execution Evidence\API-AUTH-004.png</x:v>
       </x:c>
       <x:c r="W17" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X17" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" s="47" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="B18" s="50" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="B18" s="50" t="s">
+      <x:c r="C18" s="47" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="F18" s="46" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="C18" s="47" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D18" s="47" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E18" s="47" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="F18" s="46" t="s">
+      <x:c r="G18" s="47" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H18" s="47" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="G18" s="47" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="H18" s="47" t="s">
+      <x:c r="I18" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J18" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K18" s="46" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="I18" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J18" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K18" s="46" t="s">
+      <x:c r="L18" s="46" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="L18" s="46" t="s">
+      <x:c r="M18" s="46" t="s">
         <x:v>110</x:v>
-      </x:c>
-      <x:c r="M18" s="46" t="s">
-        <x:v>111</x:v>
       </x:c>
       <x:c r="N18" s="47">
         <x:v>200</x:v>
@@ -3051,7 +3068,7 @@
         <x:v>200 transport | responseCode 201 | User created!</x:v>
       </x:c>
       <x:c r="R18" s="47" t="n">
-        <x:v>391</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="S18" s="47" t="str">
         <x:v>Pass</x:v>
@@ -3060,58 +3077,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U18" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V18" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-001.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-ACCOUNT-001.png
 ..\..\Automation\Execution Evidence\API-ACCOUNT-001.png</x:v>
       </x:c>
       <x:c r="W18" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X18" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" s="47" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="B19" s="50" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="B19" s="50" t="s">
+      <x:c r="C19" s="47" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D19" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E19" s="47" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="F19" s="46" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="C19" s="47" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D19" s="47" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E19" s="47" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="F19" s="46" t="s">
+      <x:c r="G19" s="47" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="H19" s="47" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="G19" s="47" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="H19" s="47" t="s">
+      <x:c r="I19" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J19" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K19" s="46" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I19" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J19" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K19" s="46" t="s">
+      <x:c r="L19" s="46" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="L19" s="46" t="s">
+      <x:c r="M19" s="46" t="s">
         <x:v>117</x:v>
-      </x:c>
-      <x:c r="M19" s="46" t="s">
-        <x:v>118</x:v>
       </x:c>
       <x:c r="N19" s="47">
         <x:v>200</x:v>
@@ -3126,7 +3145,7 @@
         <x:v>200 transport | responseCode 200 | Account deleted!</x:v>
       </x:c>
       <x:c r="R19" s="47" t="n">
-        <x:v>481</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="S19" s="47" t="str">
         <x:v>Pass</x:v>
@@ -3135,58 +3154,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U19" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V19" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-002.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-ACCOUNT-002.png
 ..\..\Automation\Execution Evidence\API-ACCOUNT-002.png</x:v>
       </x:c>
       <x:c r="W19" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X19" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" s="47" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B20" s="50" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="B20" s="50" t="s">
+      <x:c r="C20" s="47" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E20" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F20" s="46" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="C20" s="47" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D20" s="47" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E20" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F20" s="46" t="s">
+      <x:c r="G20" s="47" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="H20" s="47" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="G20" s="47" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="H20" s="47" t="s">
+      <x:c r="I20" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J20" s="47" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="K20" s="46" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="I20" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J20" s="47" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K20" s="46" t="s">
+      <x:c r="L20" s="46" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="M20" s="46" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="L20" s="46" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="M20" s="46" t="s">
-        <x:v>124</x:v>
       </x:c>
       <x:c r="N20" s="47">
         <x:v>200</x:v>
@@ -3201,7 +3222,7 @@
         <x:v>200 transport | responseCode 200 | User updated!</x:v>
       </x:c>
       <x:c r="R20" s="47" t="n">
-        <x:v>379</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="S20" s="47" t="str">
         <x:v>Pass</x:v>
@@ -3210,58 +3231,60 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U20" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V20" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-003.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-ACCOUNT-003.png
 ..\..\Automation\Execution Evidence\API-ACCOUNT-003.png</x:v>
       </x:c>
       <x:c r="W20" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X20" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" s="47" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="B21" s="50" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="B21" s="50" t="s">
+      <x:c r="C21" s="47" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E21" s="47" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F21" s="46" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="C21" s="47" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D21" s="47" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E21" s="47" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F21" s="46" t="s">
+      <x:c r="G21" s="47" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="H21" s="47" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="G21" s="47" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="H21" s="47" t="s">
+      <x:c r="I21" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="J21" s="47" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="K21" s="46" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="I21" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="J21" s="47" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="K21" s="46" t="s">
+      <x:c r="L21" s="46" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="L21" s="46" t="s">
+      <x:c r="M21" s="46" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="M21" s="46" t="s">
-        <x:v>131</x:v>
       </x:c>
       <x:c r="N21" s="47">
         <x:v>200</x:v>
@@ -3276,7 +3299,7 @@
         <x:v>200 transport | responseCode 200 | user detail returned</x:v>
       </x:c>
       <x:c r="R21" s="47" t="n">
-        <x:v>358</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="S21" s="47" t="str">
         <x:v>Pass</x:v>
@@ -3285,17 +3308,19 @@
         <x:v>KM</x:v>
       </x:c>
       <x:c r="U21" s="49" t="n">
-        <x:v>46239</x:v>
+        <x:v>46243</x:v>
       </x:c>
       <x:c r="V21" s="54" t="str">
-        <x:v>..\Execution Results\Screenshots\API-ACCOUNT-004.png
+        <x:v>..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md
+..\Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json
+..\Execution Results\Screenshots\API-ACCOUNT-004.png
 ..\..\Automation\Execution Evidence\API-ACCOUNT-004.png</x:v>
       </x:c>
       <x:c r="W21" s="47" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="X21" s="57" t="str">
-        <x:v>Current automated verification passed. Historical Postman runner evidence is retained as the execution baseline.</x:v>
+        <x:v>Fresh Postman collection run passed 3/3 assertions on 2026-08-09. Independent Playwright verification also passed. Historical August 1 evidence remains retained separately.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3318,7 +3343,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4830e1dfce18425c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb97224d8f2340d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3336,7 +3361,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="11" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B1" s="11"/>
       <x:c r="C1" s="11"/>
@@ -3348,7 +3373,7 @@
     </x:row>
     <x:row r="3" ht="15.5">
       <x:c r="A3" s="44" t="s">
-        <x:v>133</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B3" s="44"/>
       <x:c r="C3" s="44"/>
@@ -3428,83 +3453,83 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="B11" s="6" t="s">
+      <x:c r="C11" s="6" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="C11" s="6" t="s">
+      <x:c r="D11" s="7" t="s">
         <x:v>136</x:v>
-      </x:c>
-      <x:c r="D11" s="7" t="s">
-        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="47" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B12" s="47" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="C12" s="47" t="s">
+      <x:c r="D12" s="47" t="s">
         <x:v>139</x:v>
-      </x:c>
-      <x:c r="D12" s="47" t="s">
-        <x:v>140</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="47" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B13" s="47" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="C13" s="47" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="s">
         <x:v>141</x:v>
-      </x:c>
-      <x:c r="D13" s="47" t="s">
-        <x:v>142</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="47" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="B14" s="47" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="B14" s="47" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="C14" s="47" t="s">
+      <x:c r="D14" s="47" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="D14" s="47" t="s">
-        <x:v>145</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="47" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B15" s="47" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="C15" s="47" t="s">
+      <x:c r="D15" s="47" t="s">
         <x:v>147</x:v>
-      </x:c>
-      <x:c r="D15" s="47" t="s">
-        <x:v>148</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="47" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B16" s="47" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="C16" s="47" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D16" s="47" t="str">
         <x:v>Use HTTP 200 for this application. Record the official scenario code inside Expected Response as the JSON responseCode.</x:v>
@@ -3512,100 +3537,100 @@
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="47" t="s">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B17" s="47" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="s">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="C17" s="47" t="s">
+      <x:c r="D17" s="47" t="s">
         <x:v>151</x:v>
-      </x:c>
-      <x:c r="D17" s="47" t="s">
-        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="47" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B18" s="47" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="C18" s="47" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="s">
         <x:v>153</x:v>
-      </x:c>
-      <x:c r="D18" s="47" t="s">
-        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="47" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="B19" s="47" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="C19" s="47" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="B19" s="47" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="C19" s="47" t="s">
+      <x:c r="D19" s="47" t="s">
         <x:v>156</x:v>
-      </x:c>
-      <x:c r="D19" s="47" t="s">
-        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="47" t="s">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B20" s="47" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="C20" s="47" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="s">
         <x:v>158</x:v>
-      </x:c>
-      <x:c r="D20" s="47" t="s">
-        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="47" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="B21" s="47" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="C21" s="47" t="s">
         <x:v>160</x:v>
       </x:c>
-      <x:c r="B21" s="47" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="C21" s="47" t="s">
+      <x:c r="D21" s="47" t="s">
         <x:v>161</x:v>
-      </x:c>
-      <x:c r="D21" s="47" t="s">
-        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="47" t="s">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B22" s="47" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="C22" s="47" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="C22" s="47" t="s">
+      <x:c r="D22" s="47" t="s">
         <x:v>164</x:v>
-      </x:c>
-      <x:c r="D22" s="47" t="s">
-        <x:v>165</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="47" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B23" s="47" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="C23" s="47" t="s">
         <x:v>166</x:v>
       </x:c>
-      <x:c r="C23" s="47" t="s">
+      <x:c r="D23" s="47" t="s">
         <x:v>167</x:v>
-      </x:c>
-      <x:c r="D23" s="47" t="s">
-        <x:v>168</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3631,19 +3656,19 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="8" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="B1" s="9" t="s">
+      <x:c r="C1" s="9" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="C1" s="9" t="s">
+      <x:c r="D1" s="9" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="D1" s="9" t="s">
+      <x:c r="E1" s="10" t="s">
         <x:v>172</x:v>
-      </x:c>
-      <x:c r="E1" s="10" t="s">
-        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -3651,13 +3676,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="48" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C2" s="48" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D2" s="48" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E2" s="48" t="s">
         <x:v>4</x:v>
@@ -3665,60 +3690,60 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="48" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="48" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C3" s="48" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D3" s="48" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="E3" s="48" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="48" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="48"/>
       <x:c r="C4" s="48" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D4" s="48" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E4" s="48" t="s">
-        <x:v>175</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="48" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="48"/>
       <x:c r="C5" s="48" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="D5" s="48" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="E5" s="48" t="s">
         <x:v>176</x:v>
-      </x:c>
-      <x:c r="D5" s="48" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="E5" s="48" t="s">
-        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="48" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="48"/>
       <x:c r="C6" s="48"/>
       <x:c r="D6" s="48"/>
       <x:c r="E6" s="48" t="s">
-        <x:v>178</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3754,7 +3779,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="77" t="str">
-        <x:v>Reconciled 2026-08-09 | authoritative requirements, Postman baseline, current verification, evidence, and defect disposition</x:v>
+        <x:v>Reconciled 2026-08-09 | clean Postman execution, independent Playwright verification, historical baseline, evidence, and defect disposition</x:v>
       </x:c>
       <x:c r="B2" s="77"/>
       <x:c r="C2" s="77"/>
@@ -3796,27 +3821,27 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="78" t="str">
-        <x:v>Historical Postman baseline</x:v>
+        <x:v>Clean Postman runner</x:v>
       </x:c>
       <x:c r="B5" s="78" t="str">
-        <x:v>37 assertions | 28 passed | 9 failed | 2 runner errors</x:v>
+        <x:v>14 requests | 42 assertions | 42 passed | 0 failed | 0 errors</x:v>
       </x:c>
       <x:c r="C5" s="78"/>
       <x:c r="D5" s="78"/>
       <x:c r="E5" s="78"/>
       <x:c r="F5" s="78" t="str">
-        <x:v>Postman runner</x:v>
+        <x:v>Clean Postman run</x:v>
       </x:c>
       <x:c r="G5" s="78" t="str">
-        <x:v>Historical execution baseline</x:v>
+        <x:v>Current 42/42 verification</x:v>
       </x:c>
       <x:c r="H5" s="78" t="str">
-        <x:v>Execution Results\Postman Reports</x:v>
+        <x:v>Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09-Run-Summary.md</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="78" t="str">
-        <x:v>Current automated verification</x:v>
+        <x:v>Current Playwright verification</x:v>
       </x:c>
       <x:c r="B6" s="78" t="str">
         <x:v>14 of 14 canonical API scenarios passed</x:v>
@@ -3825,21 +3850,21 @@
       <x:c r="D6" s="78"/>
       <x:c r="E6" s="78"/>
       <x:c r="F6" s="78" t="str">
-        <x:v>Postman screenshots</x:v>
+        <x:v>Reconstructed run JSON</x:v>
       </x:c>
       <x:c r="G6" s="78" t="str">
-        <x:v>Request and response evidence</x:v>
+        <x:v>Request-level runner record</x:v>
       </x:c>
       <x:c r="H6" s="78" t="str">
-        <x:v>Execution Results\Screenshots</x:v>
+        <x:v>Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-09.reconstructed.postman_run.json</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="78" t="str">
-        <x:v>Open confirmed API defects</x:v>
+        <x:v>Historical Postman baseline</x:v>
       </x:c>
       <x:c r="B7" s="78" t="str">
-        <x:v>0</x:v>
+        <x:v>37 assertions | 28 passed | 9 failed | 2 runner errors</x:v>
       </x:c>
       <x:c r="C7" s="78"/>
       <x:c r="D7" s="78"/>
@@ -3848,7 +3873,7 @@
         <x:v>Playwright API validation</x:v>
       </x:c>
       <x:c r="G7" s="78" t="str">
-        <x:v>Current independent verification</x:v>
+        <x:v>Independent current verification</x:v>
       </x:c>
       <x:c r="H7" s="78" t="str">
         <x:v>..\..\Automation\Execution Evidence</x:v>
@@ -3856,17 +3881,23 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="78" t="str">
-        <x:v>Rejected configuration defects</x:v>
+        <x:v>API defect disposition</x:v>
       </x:c>
       <x:c r="B8" s="78" t="str">
-        <x:v>BUG-API-001 | BUG-API-002</x:v>
+        <x:v>0 open | 2 rejected: BUG-API-001, BUG-API-002</x:v>
       </x:c>
       <x:c r="C8" s="78"/>
       <x:c r="D8" s="78"/>
       <x:c r="E8" s="78"/>
-      <x:c r="F8" s="78"/>
-      <x:c r="G8" s="78"/>
-      <x:c r="H8" s="78"/>
+      <x:c r="F8" s="78" t="str">
+        <x:v>Historical Postman baseline</x:v>
+      </x:c>
+      <x:c r="G8" s="78" t="str">
+        <x:v>Audit and reconciliation history</x:v>
+      </x:c>
+      <x:c r="H8" s="78" t="str">
+        <x:v>Execution Results\Postman Reports\AE-API_Full-Collection_QA_2026-08-01-Run-Summary.md</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="78"/>
@@ -4010,7 +4041,7 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="81" t="str">
-        <x:v>Automation Exercise returns HTTP transport status 200 for these endpoints and places the documented business result in the JSON responseCode field. The historical Postman failures were retained for auditability, then reconciled against the official API specification and current automated evidence. They do not represent nine confirmed product defects.</x:v>
+        <x:v>Automation Exercise returns HTTP transport status 200 for these endpoints and places the documented scenario result in the JSON responseCode field. The corrected Postman collection now verifies both layers independently. The clean 2026-08-09 run passed 42 of 42 assertions; the 2026-08-01 failures remain preserved as historical test-script, credential, and configuration evidence rather than confirmed product defects.</x:v>
       </x:c>
       <x:c r="B18" s="81"/>
       <x:c r="C18" s="81"/>
@@ -4052,7 +4083,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="82" t="str">
-        <x:v>QA sign-off | all 14 official API requirements are traceable, executed, evidenced, and currently passing. The Postman collection should be rerun after assertion updates whenever the service changes.</x:v>
+        <x:v>QA sign-off | all 14 official API requirements are traceable, executed, evidenced, and currently passing in both Postman and Playwright. Clean Postman run: 42/42 assertions passed on 2026-08-09 with zero errors.</x:v>
       </x:c>
       <x:c r="B22" s="82"/>
       <x:c r="C22" s="82"/>

</xml_diff>